<commit_message>
fix cod art 3.1
</commit_message>
<xml_diff>
--- a/backend/upload/templates/report-templates/report_GZ.xlsx
+++ b/backend/upload/templates/report-templates/report_GZ.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="126">
   <si>
     <t xml:space="preserve">Часть I. Сведения об оказываемых государственных услугах </t>
   </si>
@@ -426,6 +426,10 @@
   <si>
     <t>3. Доля обучающихся, принявших участие в мероприятиях не ниже регионального уровня, в общем числе обучающихся</t>
   </si>
+  <si>
+    <t>3. Результативность достижений учащихся:
+3.1. Доля победителей и призеров конкурсов не ниже регионального уровня в числе обучающихся, ставших заявленными участниками</t>
+  </si>
 </sst>
 </file>
 
@@ -823,6 +827,27 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -835,41 +860,23 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -908,13 +915,13 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -967,15 +974,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -985,8 +983,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1282,22 +1286,22 @@
   <sheetData>
     <row r="1" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="59" t="s">
         <v>91</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
     </row>
     <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="59" t="s">
         <v>92</v>
       </c>
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
     </row>
     <row r="4" spans="1:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="29" t="s">
@@ -1321,11 +1325,11 @@
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="53" t="s">
+      <c r="A9" s="50" t="s">
         <v>96</v>
       </c>
-      <c r="B9" s="53"/>
-      <c r="D9" s="58" t="s">
+      <c r="B9" s="50"/>
+      <c r="D9" s="53" t="s">
         <v>104</v>
       </c>
       <c r="E9" s="27" t="s">
@@ -1337,7 +1341,7 @@
         <v>97</v>
       </c>
       <c r="B10" s="54"/>
-      <c r="D10" s="58"/>
+      <c r="D10" s="53"/>
       <c r="E10" s="27">
         <v>506501</v>
       </c>
@@ -1355,26 +1359,26 @@
     <row r="12" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="54"/>
       <c r="B12" s="54"/>
-      <c r="D12" s="58" t="s">
+      <c r="D12" s="53" t="s">
         <v>106</v>
       </c>
-      <c r="E12" s="49" t="s">
+      <c r="E12" s="56" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="54"/>
       <c r="B13" s="54"/>
-      <c r="D13" s="58"/>
-      <c r="E13" s="50"/>
+      <c r="D13" s="53"/>
+      <c r="E13" s="57"/>
     </row>
     <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="54" t="s">
         <v>99</v>
       </c>
       <c r="B14" s="54"/>
-      <c r="D14" s="58"/>
-      <c r="E14" s="51"/>
+      <c r="D14" s="53"/>
+      <c r="E14" s="58"/>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="55" t="s">
@@ -1413,35 +1417,41 @@
       <c r="E18" s="32"/>
     </row>
     <row r="19" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="53"/>
-      <c r="B19" s="53"/>
+      <c r="A19" s="50"/>
+      <c r="B19" s="50"/>
       <c r="D19" s="36" t="s">
         <v>107</v>
       </c>
       <c r="E19" s="32"/>
     </row>
     <row r="20" spans="1:5" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="56" t="s">
+      <c r="A20" s="51" t="s">
         <v>101</v>
       </c>
-      <c r="B20" s="56"/>
+      <c r="B20" s="51"/>
       <c r="E20" s="32"/>
     </row>
     <row r="21" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="57" t="s">
+      <c r="A21" s="52" t="s">
         <v>102</v>
       </c>
-      <c r="B21" s="57"/>
+      <c r="B21" s="52"/>
       <c r="E21" s="32"/>
     </row>
     <row r="22" spans="1:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="56" t="s">
+      <c r="A22" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="B22" s="56"/>
+      <c r="B22" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A21:B21"/>
@@ -1455,12 +1465,6 @@
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A12:B12"/>
-    <mergeCell ref="E12:E14"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1487,22 +1491,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="64" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="63"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
+      <c r="I1" s="64"/>
+      <c r="J1" s="64"/>
+      <c r="K1" s="64"/>
+      <c r="L1" s="64"/>
+      <c r="M1" s="64"/>
+      <c r="N1" s="65"/>
     </row>
     <row r="2" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G2" s="4" t="s">
@@ -1515,164 +1519,164 @@
       <c r="N3" s="1"/>
     </row>
     <row r="4" spans="1:17" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="67" t="s">
+      <c r="A4" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="67"/>
-      <c r="C4" s="67"/>
-      <c r="D4" s="68" t="s">
+      <c r="B4" s="68"/>
+      <c r="C4" s="68"/>
+      <c r="D4" s="69" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="76" t="s">
+      <c r="E4" s="69"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="69"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="69"/>
+      <c r="J4" s="69"/>
+      <c r="K4" s="77" t="s">
         <v>8</v>
       </c>
-      <c r="L4" s="76"/>
-      <c r="M4" s="70" t="s">
+      <c r="L4" s="77"/>
+      <c r="M4" s="71" t="s">
         <v>9</v>
       </c>
-      <c r="N4" s="71"/>
+      <c r="N4" s="72"/>
     </row>
     <row r="5" spans="1:17" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K5" s="76"/>
-      <c r="L5" s="76"/>
-      <c r="M5" s="72"/>
-      <c r="N5" s="73"/>
+      <c r="K5" s="77"/>
+      <c r="L5" s="77"/>
+      <c r="M5" s="73"/>
+      <c r="N5" s="74"/>
     </row>
     <row r="6" spans="1:17" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="67" t="s">
+      <c r="A6" s="68" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="67"/>
-      <c r="C6" s="67"/>
-      <c r="D6" s="68" t="s">
+      <c r="B6" s="68"/>
+      <c r="C6" s="68"/>
+      <c r="D6" s="69" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="68"/>
-      <c r="F6" s="68"/>
-      <c r="G6" s="68"/>
-      <c r="H6" s="68"/>
-      <c r="I6" s="68"/>
-      <c r="J6" s="68"/>
-      <c r="K6" s="76"/>
-      <c r="L6" s="76"/>
-      <c r="M6" s="72"/>
-      <c r="N6" s="73"/>
+      <c r="E6" s="69"/>
+      <c r="F6" s="69"/>
+      <c r="G6" s="69"/>
+      <c r="H6" s="69"/>
+      <c r="I6" s="69"/>
+      <c r="J6" s="69"/>
+      <c r="K6" s="77"/>
+      <c r="L6" s="77"/>
+      <c r="M6" s="73"/>
+      <c r="N6" s="74"/>
     </row>
     <row r="7" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D7" s="69"/>
-      <c r="E7" s="69"/>
-      <c r="F7" s="69"/>
-      <c r="G7" s="69"/>
-      <c r="H7" s="69"/>
-      <c r="I7" s="69"/>
-      <c r="J7" s="69"/>
-      <c r="K7" s="76"/>
-      <c r="L7" s="76"/>
-      <c r="M7" s="74"/>
-      <c r="N7" s="75"/>
+      <c r="D7" s="70"/>
+      <c r="E7" s="70"/>
+      <c r="F7" s="70"/>
+      <c r="G7" s="70"/>
+      <c r="H7" s="70"/>
+      <c r="I7" s="70"/>
+      <c r="J7" s="70"/>
+      <c r="K7" s="77"/>
+      <c r="L7" s="77"/>
+      <c r="M7" s="75"/>
+      <c r="N7" s="76"/>
     </row>
     <row r="8" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N8" s="1"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="65" t="s">
+      <c r="A9" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="65"/>
-      <c r="C9" s="65"/>
-      <c r="D9" s="65"/>
-      <c r="E9" s="65"/>
-      <c r="F9" s="65"/>
-      <c r="G9" s="65"/>
-      <c r="H9" s="65"/>
-      <c r="I9" s="65"/>
-      <c r="J9" s="65"/>
-      <c r="K9" s="65"/>
-      <c r="L9" s="65"/>
-      <c r="M9" s="65"/>
-      <c r="N9" s="66"/>
+      <c r="B9" s="66"/>
+      <c r="C9" s="66"/>
+      <c r="D9" s="66"/>
+      <c r="E9" s="66"/>
+      <c r="F9" s="66"/>
+      <c r="G9" s="66"/>
+      <c r="H9" s="66"/>
+      <c r="I9" s="66"/>
+      <c r="J9" s="66"/>
+      <c r="K9" s="66"/>
+      <c r="L9" s="66"/>
+      <c r="M9" s="66"/>
+      <c r="N9" s="67"/>
     </row>
     <row r="10" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="65" t="s">
+      <c r="A10" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="65"/>
-      <c r="C10" s="65"/>
-      <c r="D10" s="65"/>
-      <c r="E10" s="65"/>
-      <c r="F10" s="65"/>
-      <c r="G10" s="65"/>
-      <c r="H10" s="65"/>
-      <c r="I10" s="65"/>
-      <c r="J10" s="65"/>
-      <c r="K10" s="65"/>
-      <c r="L10" s="65"/>
-      <c r="M10" s="65"/>
-      <c r="N10" s="66"/>
+      <c r="B10" s="66"/>
+      <c r="C10" s="66"/>
+      <c r="D10" s="66"/>
+      <c r="E10" s="66"/>
+      <c r="F10" s="66"/>
+      <c r="G10" s="66"/>
+      <c r="H10" s="66"/>
+      <c r="I10" s="66"/>
+      <c r="J10" s="66"/>
+      <c r="K10" s="66"/>
+      <c r="L10" s="66"/>
+      <c r="M10" s="66"/>
+      <c r="N10" s="67"/>
     </row>
     <row r="11" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N11" s="1"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" s="64" t="s">
+      <c r="A12" s="63" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="64" t="s">
+      <c r="B12" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="77"/>
-      <c r="D12" s="77"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
       <c r="E12" s="78" t="s">
         <v>15</v>
       </c>
-      <c r="F12" s="79"/>
-      <c r="G12" s="79" t="s">
+      <c r="F12" s="61"/>
+      <c r="G12" s="61" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="79"/>
-      <c r="I12" s="79"/>
-      <c r="J12" s="79"/>
-      <c r="K12" s="79"/>
-      <c r="L12" s="79"/>
-      <c r="M12" s="79"/>
-      <c r="N12" s="79"/>
+      <c r="H12" s="61"/>
+      <c r="I12" s="61"/>
+      <c r="J12" s="61"/>
+      <c r="K12" s="61"/>
+      <c r="L12" s="61"/>
+      <c r="M12" s="61"/>
+      <c r="N12" s="61"/>
     </row>
     <row r="13" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="64"/>
-      <c r="B13" s="77"/>
-      <c r="C13" s="77"/>
-      <c r="D13" s="77"/>
-      <c r="E13" s="79"/>
-      <c r="F13" s="79"/>
-      <c r="G13" s="77" t="s">
+      <c r="A13" s="63"/>
+      <c r="B13" s="62"/>
+      <c r="C13" s="62"/>
+      <c r="D13" s="62"/>
+      <c r="E13" s="61"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="H13" s="64" t="s">
+      <c r="H13" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="77"/>
-      <c r="J13" s="77" t="s">
+      <c r="I13" s="62"/>
+      <c r="J13" s="62" t="s">
         <v>23</v>
       </c>
-      <c r="K13" s="77"/>
-      <c r="L13" s="64" t="s">
+      <c r="K13" s="62"/>
+      <c r="L13" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="M13" s="64" t="s">
+      <c r="M13" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="N13" s="64" t="s">
+      <c r="N13" s="63" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:17" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="64"/>
+      <c r="A14" s="63"/>
       <c r="B14" s="8" t="s">
         <v>12</v>
       </c>
@@ -1688,7 +1692,7 @@
       <c r="F14" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="77"/>
+      <c r="G14" s="62"/>
       <c r="H14" s="9" t="s">
         <v>21</v>
       </c>
@@ -1701,9 +1705,9 @@
       <c r="K14" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="L14" s="64"/>
-      <c r="M14" s="77"/>
-      <c r="N14" s="64"/>
+      <c r="L14" s="63"/>
+      <c r="M14" s="62"/>
+      <c r="N14" s="63"/>
     </row>
     <row r="15" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6">
@@ -1753,22 +1757,22 @@
       <c r="Q15" s="3"/>
     </row>
     <row r="16" spans="1:17" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="59" t="s">
+      <c r="A16" s="60" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="59" t="s">
+      <c r="B16" s="60" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="59" t="s">
+      <c r="C16" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="59" t="s">
+      <c r="D16" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="E16" s="59" t="s">
+      <c r="E16" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="F16" s="59" t="s">
+      <c r="F16" s="60" t="s">
         <v>34</v>
       </c>
       <c r="G16" s="12" t="s">
@@ -1791,12 +1795,12 @@
       <c r="N16" s="11"/>
     </row>
     <row r="17" spans="1:14" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="59"/>
-      <c r="B17" s="59"/>
-      <c r="C17" s="59"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="59"/>
-      <c r="F17" s="59"/>
+      <c r="A17" s="60"/>
+      <c r="B17" s="60"/>
+      <c r="C17" s="60"/>
+      <c r="D17" s="60"/>
+      <c r="E17" s="60"/>
+      <c r="F17" s="60"/>
       <c r="G17" s="12" t="s">
         <v>36</v>
       </c>
@@ -1895,22 +1899,22 @@
       <c r="N20" s="5"/>
     </row>
     <row r="21" spans="1:14" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="59" t="s">
+      <c r="A21" s="60" t="s">
         <v>43</v>
       </c>
-      <c r="B21" s="59" t="s">
+      <c r="B21" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="59" t="s">
+      <c r="C21" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="D21" s="59" t="s">
+      <c r="D21" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="E21" s="59" t="s">
+      <c r="E21" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="F21" s="59" t="s">
+      <c r="F21" s="60" t="s">
         <v>34</v>
       </c>
       <c r="G21" s="12" t="s">
@@ -1933,12 +1937,12 @@
       <c r="N21" s="5"/>
     </row>
     <row r="22" spans="1:14" ht="95.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="59"/>
-      <c r="B22" s="59"/>
-      <c r="C22" s="59"/>
-      <c r="D22" s="59"/>
-      <c r="E22" s="59"/>
-      <c r="F22" s="59"/>
+      <c r="A22" s="60"/>
+      <c r="B22" s="60"/>
+      <c r="C22" s="60"/>
+      <c r="D22" s="60"/>
+      <c r="E22" s="60"/>
+      <c r="F22" s="60"/>
       <c r="G22" s="12" t="s">
         <v>36</v>
       </c>
@@ -2011,22 +2015,22 @@
       <c r="N24" s="5"/>
     </row>
     <row r="25" spans="1:14" ht="96" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="59" t="s">
+      <c r="A25" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="B25" s="59" t="s">
+      <c r="B25" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="C25" s="59" t="s">
+      <c r="C25" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="D25" s="59" t="s">
+      <c r="D25" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="E25" s="59" t="s">
+      <c r="E25" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="F25" s="59" t="s">
+      <c r="F25" s="60" t="s">
         <v>34</v>
       </c>
       <c r="G25" s="12" t="s">
@@ -2049,12 +2053,12 @@
       <c r="N25" s="5"/>
     </row>
     <row r="26" spans="1:14" ht="107.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="59"/>
-      <c r="B26" s="59"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="59"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="59"/>
+      <c r="A26" s="60"/>
+      <c r="B26" s="60"/>
+      <c r="C26" s="60"/>
+      <c r="D26" s="60"/>
+      <c r="E26" s="60"/>
+      <c r="F26" s="60"/>
       <c r="G26" s="12" t="s">
         <v>36</v>
       </c>
@@ -2127,22 +2131,22 @@
       <c r="N28" s="5"/>
     </row>
     <row r="29" spans="1:14" ht="113.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="59" t="s">
+      <c r="A29" s="60" t="s">
         <v>49</v>
       </c>
-      <c r="B29" s="59" t="s">
+      <c r="B29" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="C29" s="59" t="s">
+      <c r="C29" s="60" t="s">
         <v>50</v>
       </c>
-      <c r="D29" s="59" t="s">
+      <c r="D29" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="E29" s="59" t="s">
+      <c r="E29" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="F29" s="59" t="s">
+      <c r="F29" s="60" t="s">
         <v>34</v>
       </c>
       <c r="G29" s="12" t="s">
@@ -2165,12 +2169,12 @@
       <c r="N29" s="5"/>
     </row>
     <row r="30" spans="1:14" ht="105" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="59"/>
-      <c r="B30" s="59"/>
-      <c r="C30" s="59"/>
-      <c r="D30" s="59"/>
-      <c r="E30" s="59"/>
-      <c r="F30" s="59"/>
+      <c r="A30" s="60"/>
+      <c r="B30" s="60"/>
+      <c r="C30" s="60"/>
+      <c r="D30" s="60"/>
+      <c r="E30" s="60"/>
+      <c r="F30" s="60"/>
       <c r="G30" s="12" t="s">
         <v>36</v>
       </c>
@@ -2243,22 +2247,22 @@
       <c r="N32" s="5"/>
     </row>
     <row r="33" spans="1:14" ht="192.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="59" t="s">
+      <c r="A33" s="60" t="s">
         <v>43</v>
       </c>
-      <c r="B33" s="59" t="s">
+      <c r="B33" s="60" t="s">
         <v>51</v>
       </c>
-      <c r="C33" s="59" t="s">
+      <c r="C33" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="D33" s="59" t="s">
+      <c r="D33" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="E33" s="59" t="s">
+      <c r="E33" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="F33" s="59" t="s">
+      <c r="F33" s="60" t="s">
         <v>34</v>
       </c>
       <c r="G33" s="12" t="s">
@@ -2281,12 +2285,12 @@
       <c r="N33" s="5"/>
     </row>
     <row r="34" spans="1:14" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="59"/>
-      <c r="B34" s="59"/>
-      <c r="C34" s="59"/>
-      <c r="D34" s="59"/>
-      <c r="E34" s="59"/>
-      <c r="F34" s="59"/>
+      <c r="A34" s="60"/>
+      <c r="B34" s="60"/>
+      <c r="C34" s="60"/>
+      <c r="D34" s="60"/>
+      <c r="E34" s="60"/>
+      <c r="F34" s="60"/>
       <c r="G34" s="12" t="s">
         <v>36</v>
       </c>
@@ -2385,22 +2389,22 @@
       <c r="N37" s="5"/>
     </row>
     <row r="38" spans="1:14" ht="132" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="59" t="s">
+      <c r="A38" s="60" t="s">
         <v>43</v>
       </c>
-      <c r="B38" s="59" t="s">
+      <c r="B38" s="60" t="s">
         <v>55</v>
       </c>
-      <c r="C38" s="59" t="s">
+      <c r="C38" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="D38" s="59" t="s">
+      <c r="D38" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="E38" s="59" t="s">
+      <c r="E38" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="F38" s="59" t="s">
+      <c r="F38" s="60" t="s">
         <v>34</v>
       </c>
       <c r="G38" s="12" t="s">
@@ -2423,12 +2427,12 @@
       <c r="N38" s="5"/>
     </row>
     <row r="39" spans="1:14" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="59"/>
-      <c r="B39" s="59"/>
-      <c r="C39" s="59"/>
-      <c r="D39" s="59"/>
-      <c r="E39" s="59"/>
-      <c r="F39" s="59"/>
+      <c r="A39" s="60"/>
+      <c r="B39" s="60"/>
+      <c r="C39" s="60"/>
+      <c r="D39" s="60"/>
+      <c r="E39" s="60"/>
+      <c r="F39" s="60"/>
       <c r="G39" s="12" t="s">
         <v>56</v>
       </c>
@@ -2475,22 +2479,22 @@
       <c r="N40" s="5"/>
     </row>
     <row r="41" spans="1:14" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="59" t="s">
+      <c r="A41" s="60" t="s">
         <v>111</v>
       </c>
-      <c r="B41" s="60" t="s">
+      <c r="B41" s="79" t="s">
         <v>112</v>
       </c>
-      <c r="C41" s="59" t="s">
+      <c r="C41" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="D41" s="59" t="s">
+      <c r="D41" s="60" t="s">
         <v>113</v>
       </c>
-      <c r="E41" s="59" t="s">
+      <c r="E41" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="F41" s="59" t="s">
+      <c r="F41" s="60" t="s">
         <v>34</v>
       </c>
       <c r="G41" s="42" t="s">
@@ -2513,12 +2517,12 @@
       <c r="N41" s="5"/>
     </row>
     <row r="42" spans="1:14" ht="93.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="59"/>
-      <c r="B42" s="61"/>
-      <c r="C42" s="59"/>
-      <c r="D42" s="59"/>
-      <c r="E42" s="59"/>
-      <c r="F42" s="59"/>
+      <c r="A42" s="60"/>
+      <c r="B42" s="80"/>
+      <c r="C42" s="60"/>
+      <c r="D42" s="60"/>
+      <c r="E42" s="60"/>
+      <c r="F42" s="60"/>
       <c r="G42" s="21" t="s">
         <v>36</v>
       </c>
@@ -2609,7 +2613,7 @@
       <c r="J45" s="45">
         <v>80</v>
       </c>
-      <c r="K45" s="103"/>
+      <c r="K45" s="49"/>
       <c r="L45" s="46">
         <v>0.05</v>
       </c>
@@ -2617,22 +2621,22 @@
       <c r="N45" s="43"/>
     </row>
     <row r="46" spans="1:14" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="59" t="s">
+      <c r="A46" s="60" t="s">
         <v>111</v>
       </c>
-      <c r="B46" s="60" t="s">
+      <c r="B46" s="79" t="s">
         <v>112</v>
       </c>
-      <c r="C46" s="59" t="s">
+      <c r="C46" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="D46" s="59" t="s">
+      <c r="D46" s="60" t="s">
         <v>113</v>
       </c>
-      <c r="E46" s="59" t="s">
+      <c r="E46" s="60" t="s">
         <v>114</v>
       </c>
-      <c r="F46" s="59" t="s">
+      <c r="F46" s="60" t="s">
         <v>34</v>
       </c>
       <c r="G46" s="21" t="s">
@@ -2655,12 +2659,12 @@
       <c r="N46" s="5"/>
     </row>
     <row r="47" spans="1:14" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="59"/>
-      <c r="B47" s="61"/>
-      <c r="C47" s="59"/>
-      <c r="D47" s="59"/>
-      <c r="E47" s="59"/>
-      <c r="F47" s="59"/>
+      <c r="A47" s="60"/>
+      <c r="B47" s="80"/>
+      <c r="C47" s="60"/>
+      <c r="D47" s="60"/>
+      <c r="E47" s="60"/>
+      <c r="F47" s="60"/>
       <c r="G47" s="21" t="s">
         <v>116</v>
       </c>
@@ -2849,22 +2853,22 @@
       <c r="N53" s="5"/>
     </row>
     <row r="54" spans="1:14" ht="68.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="59" t="s">
+      <c r="A54" s="60" t="s">
         <v>119</v>
       </c>
-      <c r="B54" s="60" t="s">
+      <c r="B54" s="79" t="s">
         <v>112</v>
       </c>
-      <c r="C54" s="59" t="s">
+      <c r="C54" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="D54" s="59" t="s">
+      <c r="D54" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="E54" s="59" t="s">
+      <c r="E54" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="F54" s="59" t="s">
+      <c r="F54" s="60" t="s">
         <v>34</v>
       </c>
       <c r="G54" s="21" t="s">
@@ -2887,12 +2891,12 @@
       <c r="N54" s="11"/>
     </row>
     <row r="55" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="59"/>
-      <c r="B55" s="61"/>
-      <c r="C55" s="59"/>
-      <c r="D55" s="59"/>
-      <c r="E55" s="59"/>
-      <c r="F55" s="59"/>
+      <c r="A55" s="60"/>
+      <c r="B55" s="80"/>
+      <c r="C55" s="60"/>
+      <c r="D55" s="60"/>
+      <c r="E55" s="60"/>
+      <c r="F55" s="60"/>
       <c r="G55" s="21" t="s">
         <v>36</v>
       </c>
@@ -2912,7 +2916,7 @@
       <c r="M55" s="11"/>
       <c r="N55" s="11"/>
     </row>
-    <row r="56" spans="1:14" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" ht="67.5" x14ac:dyDescent="0.25">
       <c r="A56" s="11"/>
       <c r="B56" s="11"/>
       <c r="C56" s="11"/>
@@ -2920,7 +2924,7 @@
       <c r="E56" s="11"/>
       <c r="F56" s="11"/>
       <c r="G56" s="21" t="s">
-        <v>37</v>
+        <v>125</v>
       </c>
       <c r="H56" s="13" t="s">
         <v>38</v>
@@ -2965,22 +2969,22 @@
       <c r="N57" s="5"/>
     </row>
     <row r="58" spans="1:14" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A58" s="59" t="s">
+      <c r="A58" s="60" t="s">
         <v>119</v>
       </c>
-      <c r="B58" s="60" t="s">
+      <c r="B58" s="79" t="s">
         <v>112</v>
       </c>
-      <c r="C58" s="59" t="s">
+      <c r="C58" s="60" t="s">
         <v>121</v>
       </c>
-      <c r="D58" s="59" t="s">
+      <c r="D58" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="E58" s="59" t="s">
+      <c r="E58" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="F58" s="59" t="s">
+      <c r="F58" s="60" t="s">
         <v>34</v>
       </c>
       <c r="G58" s="40" t="s">
@@ -3003,12 +3007,12 @@
       <c r="N58" s="11"/>
     </row>
     <row r="59" spans="1:14" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A59" s="59"/>
-      <c r="B59" s="61"/>
-      <c r="C59" s="59"/>
-      <c r="D59" s="59"/>
-      <c r="E59" s="59"/>
-      <c r="F59" s="59"/>
+      <c r="A59" s="60"/>
+      <c r="B59" s="80"/>
+      <c r="C59" s="60"/>
+      <c r="D59" s="60"/>
+      <c r="E59" s="60"/>
+      <c r="F59" s="60"/>
       <c r="G59" s="40" t="s">
         <v>36</v>
       </c>
@@ -3082,48 +3086,28 @@
     </row>
   </sheetData>
   <mergeCells count="80">
-    <mergeCell ref="F38:F39"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="E38:E39"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="G12:N12"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="M13:M14"/>
-    <mergeCell ref="N13:N14"/>
+    <mergeCell ref="A58:A59"/>
+    <mergeCell ref="E46:E47"/>
+    <mergeCell ref="F46:F47"/>
+    <mergeCell ref="A54:A55"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="E54:E55"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="D58:D59"/>
+    <mergeCell ref="E58:E59"/>
+    <mergeCell ref="F58:F59"/>
+    <mergeCell ref="F54:F55"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="D41:D42"/>
+    <mergeCell ref="E41:E42"/>
     <mergeCell ref="C46:C47"/>
     <mergeCell ref="D46:D47"/>
     <mergeCell ref="A1:N1"/>
@@ -3140,28 +3124,48 @@
     <mergeCell ref="K4:L7"/>
     <mergeCell ref="B12:D13"/>
     <mergeCell ref="E12:F13"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="D41:D42"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="A58:A59"/>
-    <mergeCell ref="E46:E47"/>
-    <mergeCell ref="F46:F47"/>
-    <mergeCell ref="A54:A55"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="E54:E55"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="C58:C59"/>
-    <mergeCell ref="D58:D59"/>
-    <mergeCell ref="E58:E59"/>
-    <mergeCell ref="F58:F59"/>
-    <mergeCell ref="F54:F55"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="G12:N12"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="M13:M14"/>
+    <mergeCell ref="N13:N14"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="F38:F39"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="E38:E39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="29" orientation="portrait" r:id="rId1"/>
@@ -3195,89 +3199,89 @@
   <sheetData>
     <row r="1" spans="1:15" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="80" t="s">
+      <c r="A2" s="81" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="80"/>
-      <c r="C2" s="80"/>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="80"/>
-      <c r="I2" s="80"/>
-      <c r="J2" s="80"/>
-      <c r="K2" s="80"/>
-      <c r="L2" s="80"/>
-      <c r="M2" s="80"/>
-      <c r="N2" s="80"/>
-      <c r="O2" s="80"/>
+      <c r="B2" s="81"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="81"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="81"/>
+      <c r="J2" s="81"/>
+      <c r="K2" s="81"/>
+      <c r="L2" s="81"/>
+      <c r="M2" s="81"/>
+      <c r="N2" s="81"/>
+      <c r="O2" s="81"/>
     </row>
     <row r="3" spans="1:15" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="81" t="s">
+      <c r="A4" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="84" t="s">
+      <c r="B4" s="85" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="85"/>
-      <c r="D4" s="86"/>
-      <c r="E4" s="84" t="s">
+      <c r="C4" s="86"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="85" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="86"/>
-      <c r="G4" s="64" t="s">
+      <c r="F4" s="87"/>
+      <c r="G4" s="63" t="s">
         <v>61</v>
       </c>
-      <c r="H4" s="64"/>
-      <c r="I4" s="64"/>
-      <c r="J4" s="64"/>
-      <c r="K4" s="64"/>
-      <c r="L4" s="64"/>
-      <c r="M4" s="64"/>
-      <c r="N4" s="64"/>
-      <c r="O4" s="64" t="s">
+      <c r="H4" s="63"/>
+      <c r="I4" s="63"/>
+      <c r="J4" s="63"/>
+      <c r="K4" s="63"/>
+      <c r="L4" s="63"/>
+      <c r="M4" s="63"/>
+      <c r="N4" s="63"/>
+      <c r="O4" s="63" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="82"/>
-      <c r="B5" s="87"/>
-      <c r="C5" s="88"/>
-      <c r="D5" s="89"/>
-      <c r="E5" s="87"/>
-      <c r="F5" s="89"/>
-      <c r="G5" s="64" t="s">
+      <c r="A5" s="83"/>
+      <c r="B5" s="88"/>
+      <c r="C5" s="89"/>
+      <c r="D5" s="90"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="90"/>
+      <c r="G5" s="63" t="s">
         <v>60</v>
       </c>
-      <c r="H5" s="64" t="s">
+      <c r="H5" s="63" t="s">
         <v>62</v>
       </c>
-      <c r="I5" s="64"/>
-      <c r="J5" s="64" t="s">
+      <c r="I5" s="63"/>
+      <c r="J5" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="K5" s="64"/>
-      <c r="L5" s="64" t="s">
+      <c r="K5" s="63"/>
+      <c r="L5" s="63" t="s">
         <v>66</v>
       </c>
-      <c r="M5" s="64" t="s">
+      <c r="M5" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="N5" s="64" t="s">
+      <c r="N5" s="63" t="s">
         <v>28</v>
       </c>
-      <c r="O5" s="64"/>
+      <c r="O5" s="63"/>
     </row>
     <row r="6" spans="1:15" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="83"/>
+      <c r="A6" s="84"/>
       <c r="B6" s="20"/>
       <c r="C6" s="20"/>
       <c r="D6" s="20"/>
       <c r="E6" s="20"/>
       <c r="F6" s="20"/>
-      <c r="G6" s="64"/>
+      <c r="G6" s="63"/>
       <c r="H6" s="9" t="s">
         <v>63</v>
       </c>
@@ -3290,10 +3294,10 @@
       <c r="K6" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="L6" s="64"/>
-      <c r="M6" s="64"/>
-      <c r="N6" s="64"/>
-      <c r="O6" s="64"/>
+      <c r="L6" s="63"/>
+      <c r="M6" s="63"/>
+      <c r="N6" s="63"/>
+      <c r="O6" s="63"/>
     </row>
     <row r="7" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10">
@@ -17141,22 +17145,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="64" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
+      <c r="I1" s="64"/>
+      <c r="J1" s="64"/>
+      <c r="K1" s="64"/>
+      <c r="L1" s="64"/>
+      <c r="M1" s="64"/>
+      <c r="N1" s="64"/>
     </row>
     <row r="2" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G2" s="29" t="s">
@@ -17166,11 +17170,11 @@
     </row>
     <row r="3" spans="1:14" ht="6.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="90" t="s">
+      <c r="A4" s="91" t="s">
         <v>73</v>
       </c>
-      <c r="B4" s="90"/>
-      <c r="C4" s="90"/>
+      <c r="B4" s="91"/>
+      <c r="C4" s="91"/>
       <c r="D4" s="30"/>
       <c r="E4" s="30"/>
       <c r="F4" s="30"/>
@@ -17178,25 +17182,25 @@
       <c r="H4" s="30"/>
       <c r="I4" s="30"/>
       <c r="J4" s="30"/>
-      <c r="K4" s="91" t="s">
+      <c r="K4" s="92" t="s">
         <v>8</v>
       </c>
-      <c r="L4" s="91"/>
-      <c r="M4" s="91"/>
-      <c r="N4" s="92"/>
+      <c r="L4" s="92"/>
+      <c r="M4" s="92"/>
+      <c r="N4" s="93"/>
     </row>
     <row r="5" spans="1:14" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K5" s="91"/>
-      <c r="L5" s="91"/>
-      <c r="M5" s="91"/>
-      <c r="N5" s="93"/>
+      <c r="K5" s="92"/>
+      <c r="L5" s="92"/>
+      <c r="M5" s="92"/>
+      <c r="N5" s="94"/>
     </row>
     <row r="6" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="62" t="s">
+      <c r="A6" s="64" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="62"/>
-      <c r="C6" s="62"/>
+      <c r="B6" s="64"/>
+      <c r="C6" s="64"/>
       <c r="D6" s="30"/>
       <c r="E6" s="30"/>
       <c r="F6" s="30"/>
@@ -17204,10 +17208,10 @@
       <c r="H6" s="30"/>
       <c r="I6" s="30"/>
       <c r="J6" s="30"/>
-      <c r="K6" s="91"/>
-      <c r="L6" s="91"/>
-      <c r="M6" s="91"/>
-      <c r="N6" s="93"/>
+      <c r="K6" s="92"/>
+      <c r="L6" s="92"/>
+      <c r="M6" s="92"/>
+      <c r="N6" s="94"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="31"/>
@@ -17217,109 +17221,109 @@
       <c r="H7" s="31"/>
       <c r="I7" s="31"/>
       <c r="J7" s="31"/>
-      <c r="K7" s="91"/>
-      <c r="L7" s="91"/>
-      <c r="M7" s="91"/>
-      <c r="N7" s="94"/>
+      <c r="K7" s="92"/>
+      <c r="L7" s="92"/>
+      <c r="M7" s="92"/>
+      <c r="N7" s="95"/>
     </row>
     <row r="8" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="90" t="s">
+      <c r="A9" s="91" t="s">
         <v>75</v>
       </c>
-      <c r="B9" s="90"/>
-      <c r="C9" s="90"/>
-      <c r="D9" s="90"/>
-      <c r="E9" s="90"/>
-      <c r="F9" s="90"/>
-      <c r="G9" s="90"/>
-      <c r="H9" s="90"/>
-      <c r="I9" s="90"/>
-      <c r="J9" s="90"/>
-      <c r="K9" s="90"/>
-      <c r="L9" s="90"/>
-      <c r="M9" s="90"/>
-      <c r="N9" s="90"/>
+      <c r="B9" s="91"/>
+      <c r="C9" s="91"/>
+      <c r="D9" s="91"/>
+      <c r="E9" s="91"/>
+      <c r="F9" s="91"/>
+      <c r="G9" s="91"/>
+      <c r="H9" s="91"/>
+      <c r="I9" s="91"/>
+      <c r="J9" s="91"/>
+      <c r="K9" s="91"/>
+      <c r="L9" s="91"/>
+      <c r="M9" s="91"/>
+      <c r="N9" s="91"/>
     </row>
     <row r="10" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="90" t="s">
+      <c r="A10" s="91" t="s">
         <v>76</v>
       </c>
-      <c r="B10" s="90"/>
-      <c r="C10" s="90"/>
-      <c r="D10" s="90"/>
-      <c r="E10" s="90"/>
-      <c r="F10" s="90"/>
-      <c r="G10" s="90"/>
-      <c r="H10" s="90"/>
-      <c r="I10" s="90"/>
-      <c r="J10" s="90"/>
-      <c r="K10" s="90"/>
-      <c r="L10" s="90"/>
-      <c r="M10" s="90"/>
-      <c r="N10" s="90"/>
+      <c r="B10" s="91"/>
+      <c r="C10" s="91"/>
+      <c r="D10" s="91"/>
+      <c r="E10" s="91"/>
+      <c r="F10" s="91"/>
+      <c r="G10" s="91"/>
+      <c r="H10" s="91"/>
+      <c r="I10" s="91"/>
+      <c r="J10" s="91"/>
+      <c r="K10" s="91"/>
+      <c r="L10" s="91"/>
+      <c r="M10" s="91"/>
+      <c r="N10" s="91"/>
     </row>
     <row r="11" spans="1:14" ht="10.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="81" t="s">
+      <c r="A12" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="84" t="s">
+      <c r="B12" s="85" t="s">
         <v>77</v>
       </c>
-      <c r="C12" s="85"/>
-      <c r="D12" s="86"/>
-      <c r="E12" s="84" t="s">
+      <c r="C12" s="86"/>
+      <c r="D12" s="87"/>
+      <c r="E12" s="85" t="s">
         <v>78</v>
       </c>
-      <c r="F12" s="86"/>
-      <c r="G12" s="64" t="s">
+      <c r="F12" s="87"/>
+      <c r="G12" s="63" t="s">
         <v>79</v>
       </c>
-      <c r="H12" s="64"/>
-      <c r="I12" s="64"/>
-      <c r="J12" s="64"/>
-      <c r="K12" s="64"/>
-      <c r="L12" s="64"/>
-      <c r="M12" s="64"/>
-      <c r="N12" s="64"/>
+      <c r="H12" s="63"/>
+      <c r="I12" s="63"/>
+      <c r="J12" s="63"/>
+      <c r="K12" s="63"/>
+      <c r="L12" s="63"/>
+      <c r="M12" s="63"/>
+      <c r="N12" s="63"/>
     </row>
     <row r="13" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="82"/>
-      <c r="B13" s="87"/>
-      <c r="C13" s="88"/>
-      <c r="D13" s="89"/>
-      <c r="E13" s="87"/>
-      <c r="F13" s="89"/>
-      <c r="G13" s="81" t="s">
+      <c r="A13" s="83"/>
+      <c r="B13" s="88"/>
+      <c r="C13" s="89"/>
+      <c r="D13" s="90"/>
+      <c r="E13" s="88"/>
+      <c r="F13" s="90"/>
+      <c r="G13" s="82" t="s">
         <v>19</v>
       </c>
-      <c r="H13" s="95" t="s">
+      <c r="H13" s="96" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="96"/>
-      <c r="J13" s="95" t="s">
+      <c r="I13" s="97"/>
+      <c r="J13" s="96" t="s">
         <v>23</v>
       </c>
-      <c r="K13" s="96"/>
-      <c r="L13" s="81" t="s">
+      <c r="K13" s="97"/>
+      <c r="L13" s="82" t="s">
         <v>26</v>
       </c>
-      <c r="M13" s="81" t="s">
+      <c r="M13" s="82" t="s">
         <v>27</v>
       </c>
-      <c r="N13" s="81" t="s">
+      <c r="N13" s="82" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="83"/>
+      <c r="A14" s="84"/>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
       <c r="D14" s="17"/>
       <c r="E14" s="17"/>
       <c r="F14" s="17"/>
-      <c r="G14" s="83"/>
+      <c r="G14" s="84"/>
       <c r="H14" s="17" t="s">
         <v>21</v>
       </c>
@@ -17332,9 +17336,9 @@
       <c r="K14" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="L14" s="83"/>
-      <c r="M14" s="83"/>
-      <c r="N14" s="83"/>
+      <c r="L14" s="84"/>
+      <c r="M14" s="84"/>
+      <c r="N14" s="84"/>
     </row>
     <row r="15" spans="1:14" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="17">
@@ -17381,12 +17385,12 @@
       </c>
     </row>
     <row r="16" spans="1:14" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="81"/>
-      <c r="B16" s="81"/>
-      <c r="C16" s="81"/>
-      <c r="D16" s="81"/>
-      <c r="E16" s="81"/>
-      <c r="F16" s="81"/>
+      <c r="A16" s="82"/>
+      <c r="B16" s="82"/>
+      <c r="C16" s="82"/>
+      <c r="D16" s="82"/>
+      <c r="E16" s="82"/>
+      <c r="F16" s="82"/>
       <c r="G16" s="17"/>
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
@@ -17397,12 +17401,12 @@
       <c r="N16" s="17"/>
     </row>
     <row r="17" spans="1:14" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="83"/>
-      <c r="B17" s="83"/>
-      <c r="C17" s="83"/>
-      <c r="D17" s="83"/>
-      <c r="E17" s="83"/>
-      <c r="F17" s="83"/>
+      <c r="A17" s="84"/>
+      <c r="B17" s="84"/>
+      <c r="C17" s="84"/>
+      <c r="D17" s="84"/>
+      <c r="E17" s="84"/>
+      <c r="F17" s="84"/>
       <c r="G17" s="17"/>
       <c r="H17" s="17"/>
       <c r="I17" s="17"/>
@@ -17413,12 +17417,12 @@
       <c r="N17" s="17"/>
     </row>
     <row r="18" spans="1:14" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="81"/>
-      <c r="B18" s="81"/>
-      <c r="C18" s="81"/>
-      <c r="D18" s="81"/>
-      <c r="E18" s="81"/>
-      <c r="F18" s="81"/>
+      <c r="A18" s="82"/>
+      <c r="B18" s="82"/>
+      <c r="C18" s="82"/>
+      <c r="D18" s="82"/>
+      <c r="E18" s="82"/>
+      <c r="F18" s="82"/>
       <c r="G18" s="17"/>
       <c r="H18" s="17"/>
       <c r="I18" s="17"/>
@@ -17429,12 +17433,12 @@
       <c r="N18" s="17"/>
     </row>
     <row r="19" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="83"/>
-      <c r="B19" s="83"/>
-      <c r="C19" s="83"/>
-      <c r="D19" s="83"/>
-      <c r="E19" s="83"/>
-      <c r="F19" s="83"/>
+      <c r="A19" s="84"/>
+      <c r="B19" s="84"/>
+      <c r="C19" s="84"/>
+      <c r="D19" s="84"/>
+      <c r="E19" s="84"/>
+      <c r="F19" s="84"/>
       <c r="G19" s="17"/>
       <c r="H19" s="17"/>
       <c r="I19" s="17"/>
@@ -17447,6 +17451,19 @@
     <row r="20" spans="1:14" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="M13:M14"/>
+    <mergeCell ref="N13:N14"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="F18:F19"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="K4:M7"/>
@@ -17463,19 +17480,6 @@
     <mergeCell ref="H13:I13"/>
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="L13:L14"/>
-    <mergeCell ref="M13:M14"/>
-    <mergeCell ref="N13:N14"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="F18:F19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17506,89 +17510,89 @@
   <sheetData>
     <row r="1" spans="1:15" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="90" t="s">
+      <c r="A2" s="91" t="s">
         <v>81</v>
       </c>
-      <c r="B2" s="90"/>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
-      <c r="G2" s="90"/>
-      <c r="H2" s="90"/>
-      <c r="I2" s="90"/>
-      <c r="J2" s="90"/>
-      <c r="K2" s="90"/>
-      <c r="L2" s="90"/>
-      <c r="M2" s="90"/>
-      <c r="N2" s="90"/>
-      <c r="O2" s="90"/>
+      <c r="B2" s="91"/>
+      <c r="C2" s="91"/>
+      <c r="D2" s="91"/>
+      <c r="E2" s="91"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="91"/>
+      <c r="H2" s="91"/>
+      <c r="I2" s="91"/>
+      <c r="J2" s="91"/>
+      <c r="K2" s="91"/>
+      <c r="L2" s="91"/>
+      <c r="M2" s="91"/>
+      <c r="N2" s="91"/>
+      <c r="O2" s="91"/>
     </row>
     <row r="3" spans="1:15" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="81" t="s">
+      <c r="A4" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="84" t="s">
+      <c r="B4" s="85" t="s">
         <v>77</v>
       </c>
-      <c r="C4" s="85"/>
-      <c r="D4" s="86"/>
-      <c r="E4" s="84" t="s">
+      <c r="C4" s="86"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="85" t="s">
         <v>78</v>
       </c>
-      <c r="F4" s="86"/>
-      <c r="G4" s="95" t="s">
+      <c r="F4" s="87"/>
+      <c r="G4" s="96" t="s">
         <v>82</v>
       </c>
-      <c r="H4" s="97"/>
-      <c r="I4" s="97"/>
-      <c r="J4" s="97"/>
-      <c r="K4" s="97"/>
-      <c r="L4" s="97"/>
-      <c r="M4" s="97"/>
-      <c r="N4" s="96"/>
-      <c r="O4" s="81" t="s">
+      <c r="H4" s="103"/>
+      <c r="I4" s="103"/>
+      <c r="J4" s="103"/>
+      <c r="K4" s="103"/>
+      <c r="L4" s="103"/>
+      <c r="M4" s="103"/>
+      <c r="N4" s="97"/>
+      <c r="O4" s="82" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="82"/>
-      <c r="B5" s="87"/>
-      <c r="C5" s="88"/>
-      <c r="D5" s="89"/>
-      <c r="E5" s="87"/>
-      <c r="F5" s="89"/>
-      <c r="G5" s="81" t="s">
+      <c r="A5" s="83"/>
+      <c r="B5" s="88"/>
+      <c r="C5" s="89"/>
+      <c r="D5" s="90"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="90"/>
+      <c r="G5" s="82" t="s">
         <v>60</v>
       </c>
-      <c r="H5" s="95" t="s">
+      <c r="H5" s="96" t="s">
         <v>62</v>
       </c>
-      <c r="I5" s="96"/>
-      <c r="J5" s="95" t="s">
+      <c r="I5" s="97"/>
+      <c r="J5" s="96" t="s">
         <v>23</v>
       </c>
-      <c r="K5" s="96"/>
-      <c r="L5" s="81" t="s">
+      <c r="K5" s="97"/>
+      <c r="L5" s="82" t="s">
         <v>66</v>
       </c>
-      <c r="M5" s="81" t="s">
+      <c r="M5" s="82" t="s">
         <v>27</v>
       </c>
-      <c r="N5" s="81" t="s">
+      <c r="N5" s="82" t="s">
         <v>28</v>
       </c>
-      <c r="O5" s="82"/>
+      <c r="O5" s="83"/>
     </row>
     <row r="6" spans="1:15" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="83"/>
+      <c r="A6" s="84"/>
       <c r="B6" s="20"/>
       <c r="C6" s="20"/>
       <c r="D6" s="20"/>
       <c r="E6" s="20"/>
       <c r="F6" s="20"/>
-      <c r="G6" s="83"/>
+      <c r="G6" s="84"/>
       <c r="H6" s="17" t="s">
         <v>63</v>
       </c>
@@ -17601,10 +17605,10 @@
       <c r="K6" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="L6" s="83"/>
-      <c r="M6" s="83"/>
-      <c r="N6" s="83"/>
-      <c r="O6" s="83"/>
+      <c r="L6" s="84"/>
+      <c r="M6" s="84"/>
+      <c r="N6" s="84"/>
+      <c r="O6" s="84"/>
     </row>
     <row r="7" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="17">
@@ -17654,12 +17658,12 @@
       </c>
     </row>
     <row r="8" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="81"/>
-      <c r="B8" s="81"/>
-      <c r="C8" s="81"/>
-      <c r="D8" s="81"/>
-      <c r="E8" s="81"/>
-      <c r="F8" s="81"/>
+      <c r="A8" s="82"/>
+      <c r="B8" s="82"/>
+      <c r="C8" s="82"/>
+      <c r="D8" s="82"/>
+      <c r="E8" s="82"/>
+      <c r="F8" s="82"/>
       <c r="G8" s="20"/>
       <c r="H8" s="20"/>
       <c r="I8" s="20"/>
@@ -17671,12 +17675,12 @@
       <c r="O8" s="20"/>
     </row>
     <row r="9" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="83"/>
-      <c r="B9" s="83"/>
-      <c r="C9" s="83"/>
-      <c r="D9" s="83"/>
-      <c r="E9" s="83"/>
-      <c r="F9" s="83"/>
+      <c r="A9" s="84"/>
+      <c r="B9" s="84"/>
+      <c r="C9" s="84"/>
+      <c r="D9" s="84"/>
+      <c r="E9" s="84"/>
+      <c r="F9" s="84"/>
       <c r="G9" s="20"/>
       <c r="H9" s="20"/>
       <c r="I9" s="20"/>
@@ -17688,12 +17692,12 @@
       <c r="O9" s="20"/>
     </row>
     <row r="10" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="81"/>
-      <c r="B10" s="81"/>
-      <c r="C10" s="81"/>
-      <c r="D10" s="81"/>
-      <c r="E10" s="81"/>
-      <c r="F10" s="81"/>
+      <c r="A10" s="82"/>
+      <c r="B10" s="82"/>
+      <c r="C10" s="82"/>
+      <c r="D10" s="82"/>
+      <c r="E10" s="82"/>
+      <c r="F10" s="82"/>
       <c r="G10" s="20"/>
       <c r="H10" s="20"/>
       <c r="I10" s="20"/>
@@ -17705,12 +17709,12 @@
       <c r="O10" s="20"/>
     </row>
     <row r="11" spans="1:15" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="83"/>
-      <c r="B11" s="83"/>
-      <c r="C11" s="83"/>
-      <c r="D11" s="83"/>
-      <c r="E11" s="83"/>
-      <c r="F11" s="83"/>
+      <c r="A11" s="84"/>
+      <c r="B11" s="84"/>
+      <c r="C11" s="84"/>
+      <c r="D11" s="84"/>
+      <c r="E11" s="84"/>
+      <c r="F11" s="84"/>
       <c r="G11" s="20"/>
       <c r="H11" s="20"/>
       <c r="I11" s="20"/>
@@ -17726,45 +17730,45 @@
     <row r="14" spans="1:15" ht="11.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="99" t="s">
+      <c r="A17" s="102" t="s">
         <v>84</v>
       </c>
-      <c r="B17" s="99"/>
-      <c r="C17" s="99"/>
-      <c r="D17" s="100" t="s">
+      <c r="B17" s="102"/>
+      <c r="C17" s="102"/>
+      <c r="D17" s="98" t="s">
         <v>85</v>
       </c>
-      <c r="E17" s="100"/>
-      <c r="F17" s="100"/>
-      <c r="G17" s="100"/>
-      <c r="H17" s="100"/>
-      <c r="I17" s="100"/>
-      <c r="J17" s="100"/>
-      <c r="K17" s="100" t="s">
+      <c r="E17" s="98"/>
+      <c r="F17" s="98"/>
+      <c r="G17" s="98"/>
+      <c r="H17" s="98"/>
+      <c r="I17" s="98"/>
+      <c r="J17" s="98"/>
+      <c r="K17" s="98" t="s">
         <v>89</v>
       </c>
-      <c r="L17" s="100"/>
-      <c r="M17" s="100"/>
+      <c r="L17" s="98"/>
+      <c r="M17" s="98"/>
       <c r="N17" s="26"/>
       <c r="O17" s="26"/>
     </row>
     <row r="18" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D18" s="101" t="s">
+      <c r="D18" s="99" t="s">
         <v>86</v>
       </c>
-      <c r="E18" s="101"/>
-      <c r="F18" s="101"/>
-      <c r="G18" s="101" t="s">
+      <c r="E18" s="99"/>
+      <c r="F18" s="99"/>
+      <c r="G18" s="99" t="s">
         <v>87</v>
       </c>
-      <c r="H18" s="101"/>
-      <c r="I18" s="101"/>
-      <c r="J18" s="101"/>
-      <c r="K18" s="102" t="s">
+      <c r="H18" s="99"/>
+      <c r="I18" s="99"/>
+      <c r="J18" s="99"/>
+      <c r="K18" s="100" t="s">
         <v>88</v>
       </c>
-      <c r="L18" s="102"/>
-      <c r="M18" s="102"/>
+      <c r="L18" s="100"/>
+      <c r="M18" s="100"/>
       <c r="N18" s="7"/>
       <c r="O18" s="7"/>
     </row>
@@ -17775,34 +17779,14 @@
       <c r="C20" s="30"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="98" t="s">
+      <c r="A21" s="101" t="s">
         <v>90</v>
       </c>
-      <c r="B21" s="98"/>
-      <c r="C21" s="98"/>
+      <c r="B21" s="101"/>
+      <c r="C21" s="101"/>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="K18:M18"/>
-    <mergeCell ref="K17:M17"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="F10:F11"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="B10:B11"/>
     <mergeCell ref="A2:O2"/>
     <mergeCell ref="A4:A6"/>
     <mergeCell ref="B4:D5"/>
@@ -17815,6 +17799,26 @@
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="M5:M6"/>
     <mergeCell ref="N5:N6"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="K18:M18"/>
+    <mergeCell ref="K17:M17"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="F10:F11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>